<commit_message>
replaced outdated xlsx files
</commit_message>
<xml_diff>
--- a/input/reg_eq5d.xlsx
+++ b/input/reg_eq5d.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C9A3FA-0401-C041-B79F-31750397BA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DD64083-91D2-4D92-B492-C79D07ABF086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{8A9A3AE8-34F1-4C3E-9682-3C69CFBA3626}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8A9A3AE8-34F1-4C3E-9682-3C69CFBA3626}"/>
   </bookViews>
   <sheets>
-    <sheet name="UK_EQ5D_lawrence" sheetId="1" r:id="rId1"/>
-    <sheet name="UK_EQ5D_franks" sheetId="2" r:id="rId2"/>
+    <sheet name="EQ5D_lawrence" sheetId="1" r:id="rId1"/>
+    <sheet name="EQ5D_franks" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -452,19 +452,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCCE0DF9-DC32-43B5-8DA4-440480E6714A}">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -493,7 +493,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -522,7 +522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -551,7 +551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -580,7 +580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -609,7 +609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -638,7 +638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -667,7 +667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -704,19 +704,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8079D6CA-2355-449F-ADE5-FDF6FCFCC506}">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -745,7 +745,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -774,7 +774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -803,7 +803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -832,7 +832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -861,7 +861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -890,7 +890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
restore input files to `develop` version
</commit_message>
<xml_diff>
--- a/input/reg_eq5d.xlsx
+++ b/input/reg_eq5d.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DD64083-91D2-4D92-B492-C79D07ABF086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C9A3FA-0401-C041-B79F-31750397BA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8A9A3AE8-34F1-4C3E-9682-3C69CFBA3626}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{8A9A3AE8-34F1-4C3E-9682-3C69CFBA3626}"/>
   </bookViews>
   <sheets>
-    <sheet name="EQ5D_lawrence" sheetId="1" r:id="rId1"/>
-    <sheet name="EQ5D_franks" sheetId="2" r:id="rId2"/>
+    <sheet name="UK_EQ5D_lawrence" sheetId="1" r:id="rId1"/>
+    <sheet name="UK_EQ5D_franks" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -452,19 +452,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCCE0DF9-DC32-43B5-8DA4-440480E6714A}">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -493,7 +493,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -522,7 +522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -551,7 +551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -580,7 +580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -609,7 +609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -638,7 +638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -667,7 +667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -704,19 +704,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8079D6CA-2355-449F-ADE5-FDF6FCFCC506}">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -745,7 +745,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -774,7 +774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -803,7 +803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -832,7 +832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -861,7 +861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -890,7 +890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>

</xml_diff>